<commit_message>
Prueba gratis por mensajes y recargas de +20 por $1 y +100 por $4
- La prueba se mide en mensajes (100 Personal, 200 Negocio, 300 Plus) con aviso al 80 %;
  el tope en dólares queda como red de seguridad.
- "recargar" ofrece dos recargas; el pago guarda los mensajes comprados (migración 0020).
- Modelo financiero y bitácora al día.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JDwKA1YUHPBZPD6osqPUUD
</commit_message>
<xml_diff>
--- a/docs/finanzas/rocco-modelo-financiero.xlsx
+++ b/docs/finanzas/rocco-modelo-financiero.xlsx
@@ -975,7 +975,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Recarga: precio ($)</t>
+          <t>Recarga grande: precio ($)</t>
         </is>
       </c>
       <c r="B15" s="12" t="n">
@@ -983,7 +983,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>+100 mensajes por $4 (plans.ts).</t>
+          <t>+100 mensajes por $4 (plans.ts). La chica (+20 por $1) está en la hoja Margen por plan.</t>
         </is>
       </c>
       <c r="D15" s="2" t="n"/>
@@ -993,7 +993,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Recarga: mensajes</t>
+          <t>Recarga grande: mensajes</t>
         </is>
       </c>
       <c r="B16" s="13" t="n">
@@ -1011,7 +1011,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>% de clientes que compran 1 recarga al mes</t>
+          <t>% de clientes que compran 1 recarga grande al mes</t>
         </is>
       </c>
       <c r="B17" s="14" t="n">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Supuesto: quien llega al tope y quiere seguir.</t>
+          <t>Supuesto: quien llega al tope y quiere seguir. Conservador: no cuenta las chicas.</t>
         </is>
       </c>
       <c r="D17" s="2" t="n"/>
@@ -1348,7 +1348,7 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>Prueba gratis (beta: 14 días desde el registro)</t>
+          <t>Prueba gratis (beta: 14 días desde el registro o N mensajes, lo que llegue primero)</t>
         </is>
       </c>
       <c r="B38" s="10" t="n"/>
@@ -1378,15 +1378,15 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Tope de gasto de la prueba, Personal ($)</t>
-        </is>
-      </c>
-      <c r="B40" s="12" t="n">
-        <v>1.5</v>
+          <t>Mensajes de la prueba, Personal</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="n">
+        <v>100</v>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Al llegar, Rocco deja de registrar (0016).</t>
+          <t>trialMessages en plans.ts (07/10/2026). Al pasarlos, Rocco deja de registrar.</t>
         </is>
       </c>
       <c r="D40" s="2" t="n"/>
@@ -1396,15 +1396,15 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Tope de gasto de la prueba, Negocio ($)</t>
-        </is>
-      </c>
-      <c r="B41" s="12" t="n">
-        <v>4</v>
+          <t>Mensajes de la prueba, Negocio</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="n">
+        <v>200</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Ídem.</t>
+          <t>Ídem. Plus: 300. Hay además una red de seguridad en $ (4 / 8 / 12) por si alguien manda muchas fotos.</t>
         </is>
       </c>
       <c r="D41" s="2" t="n"/>
@@ -1896,15 +1896,32 @@
       <c r="L9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="2" t="n"/>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Recarga chica (+20 mensajes)</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
+      <c r="D10" s="13" t="n">
+        <v>20</v>
+      </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
+      <c r="G10" s="26">
+        <f>D10*'Costo por mensaje'!$B$8</f>
+        <v/>
+      </c>
+      <c r="H10" s="26">
+        <f>B10*(1-Supuestos!$B$26-Supuestos!$B$27)-G10</f>
+        <v/>
+      </c>
+      <c r="I10" s="15">
+        <f>IF(B10=0,0,H10/B10)</f>
+        <v/>
+      </c>
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n"/>
@@ -3033,24 +3050,24 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Tope de gasto de la prueba ($)</t>
-        </is>
-      </c>
-      <c r="B13" s="26">
+          <t>Mensajes incluidos en la prueba</t>
+        </is>
+      </c>
+      <c r="B13" s="27">
         <f>Supuestos!B40</f>
         <v/>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="27">
         <f>Supuestos!B41</f>
         <v/>
       </c>
-      <c r="D13" s="26">
+      <c r="D13" s="27">
         <f>Supuestos!B40</f>
         <v/>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Al llegar al tope Rocco deja de registrar: ninguna prueba cuesta más.</t>
+          <t>Al pasarlos Rocco deja de registrar: ninguna prueba cuesta más.</t>
         </is>
       </c>
     </row>
@@ -3121,15 +3138,15 @@
         </is>
       </c>
       <c r="B17" s="26">
-        <f>B15*MIN(B8*'Costo por mensaje'!$B$8,B13)+B16*MIN(B9*'Costo por mensaje'!$B$8,B13)</f>
+        <f>(B15*MIN(B8,B13)+B16*MIN(B9,B13))*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
       <c r="C17" s="26">
-        <f>C15*MIN(C8*'Costo por mensaje'!$B$8,C13)+C16*MIN(C9*'Costo por mensaje'!$B$8,C13)</f>
+        <f>(C15*MIN(C8,C13)+C16*MIN(C9,C13))*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
       <c r="D17" s="26">
-        <f>D15*MIN(D8*'Costo por mensaje'!$B$8,D13)+D16*MIN(D9*'Costo por mensaje'!$B$8,D13)</f>
+        <f>(D15*MIN(D8,D13)+D16*MIN(D9,D13))*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
       <c r="E17" s="2" t="n"/>
@@ -3217,19 +3234,19 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Mensajes que alcanza el tope de la prueba</t>
-        </is>
-      </c>
-      <c r="B22" s="27">
-        <f>IF('Costo por mensaje'!$B$8=0,0,B13/'Costo por mensaje'!$B$8)</f>
-        <v/>
-      </c>
-      <c r="C22" s="27">
-        <f>IF('Costo por mensaje'!$B$8=0,0,C13/'Costo por mensaje'!$B$8)</f>
-        <v/>
-      </c>
-      <c r="D22" s="27">
-        <f>IF('Costo por mensaje'!$B$8=0,0,D13/'Costo por mensaje'!$B$8)</f>
+          <t>Costo máximo de una prueba ($)</t>
+        </is>
+      </c>
+      <c r="B22" s="26">
+        <f>B13*'Costo por mensaje'!$B$8</f>
+        <v/>
+      </c>
+      <c r="C22" s="26">
+        <f>C13*'Costo por mensaje'!$B$8</f>
+        <v/>
+      </c>
+      <c r="D22" s="26">
+        <f>D13*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
       <c r="E22" s="2" t="n"/>
@@ -3244,7 +3261,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Lectura: el tipo de persona con el CAC más bajo y más clientes que pagan es a quien debes invitar primero. Las pruebas tienen tope de gasto ($1,50 / $4), así que ninguna prueba cuesta más que eso.</t>
+          <t>Lectura: el tipo de persona con el CAC más bajo y más clientes que pagan es a quien debes invitar primero. La prueba se mide en mensajes (100 Personal / 200 Negocio): el costo máximo de una prueba está en la fila 22.</t>
         </is>
       </c>
       <c r="B24" s="2" t="n"/>
@@ -3712,7 +3729,7 @@
       </c>
       <c r="B6" s="37" t="inlineStr">
         <is>
-          <t>Lotes de 10 a 15 por semana, no 100 de una vez: así puedes acompañar a cada uno, ver en /admin quién se activa y ajustar los textos de Rocco. La prueba tiene tope de gasto: el peor caso es $1,50 por Personal y $4 por Negocio.</t>
+          <t>Lotes de 10 a 15 por semana, no 100 de una vez: así puedes acompañar a cada uno, ver en /admin quién se activa y ajustar los textos de Rocco. La prueba se mide en mensajes: el peor caso es ~$2,10 por Personal (100) y ~$4,30 por Negocio (200).</t>
         </is>
       </c>
     </row>
@@ -3755,12 +3772,12 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Ojo con el tope de la prueba Personal</t>
+          <t>Prueba por mensajes y recargas</t>
         </is>
       </c>
       <c r="B10" s="37" t="inlineStr">
         <is>
-          <t>$1,50 alcanza para unos 70 mensajes (5 por día): un usuario activo de verdad se queda sin prueba antes del día 14. Para la beta conviene subirlo a $2,50 (≈ 117 mensajes); el costo extra es de $1 por persona activa. Se cambia en /admin por negocio o en plans.ts para todos.</t>
+          <t>La prueba son 100 mensajes (Personal) o 200 (Negocio) en 14 días: unos 7 o 14 por día, más que el uso normal. Al llegar al tope del mes, quien quiere más compra recargas: +20 por $1 o +100 por $4. Las dos dejan más del 50 % de margen en el peor caso, así que el power user paga lo que usa y tu margen no cambia.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Prueba gratis única: 14 días o 100 mensajes para todos los planes
- TRIAL_MESSAGES = 100 y red de seguridad de $4 para todos; el plan se elige al pagar.
- Los mensajes regalados desde /admin suben el tope de la prueba (y la red en proporción).
- Registro web: "¿Cómo lo vas a usar?" (personal o negocio) en vez de elegir plan.
- Landing, Excel y bitácora al día.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JDwKA1YUHPBZPD6osqPUUD
</commit_message>
<xml_diff>
--- a/docs/finanzas/rocco-modelo-financiero.xlsx
+++ b/docs/finanzas/rocco-modelo-financiero.xlsx
@@ -138,6 +138,7 @@
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -151,7 +152,6 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1378,7 +1378,7 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Mensajes de la prueba, Personal</t>
+          <t>Mensajes de la prueba (única, para todos)</t>
         </is>
       </c>
       <c r="B40" s="13" t="n">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>trialMessages en plans.ts (07/10/2026). Al pasarlos, Rocco deja de registrar.</t>
+          <t>TRIAL_MESSAGES en plans.ts (07/10/2026). El plan se elige al pagar: nadie escoge Plus para tener más prueba.</t>
         </is>
       </c>
       <c r="D40" s="2" t="n"/>
@@ -1396,15 +1396,16 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Mensajes de la prueba, Negocio</t>
-        </is>
-      </c>
-      <c r="B41" s="13" t="n">
-        <v>200</v>
+          <t>Mensajes de la prueba para dueños de negocio</t>
+        </is>
+      </c>
+      <c r="B41" s="23">
+        <f>B40</f>
+        <v/>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Ídem. Plus: 300. Hay además una red de seguridad en $ (4 / 8 / 12) por si alguien manda muchas fotos.</t>
+          <t>La misma prueba. Si un negocio que vale la pena se queda corto, se le regalan +100 desde /admin (a mano).</t>
         </is>
       </c>
       <c r="D41" s="2" t="n"/>
@@ -1476,7 +1477,7 @@
           <t>IA (Anthropic)</t>
         </is>
       </c>
-      <c r="B5" s="23">
+      <c r="B5" s="24">
         <f>Supuestos!B20</f>
         <v/>
       </c>
@@ -1492,7 +1493,7 @@
           <t>Meta (respuesta de Rocco)</t>
         </is>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="24">
         <f>Supuestos!B21*Supuestos!B22</f>
         <v/>
       </c>
@@ -1508,7 +1509,7 @@
           <t>Notas de voz</t>
         </is>
       </c>
-      <c r="B7" s="23">
+      <c r="B7" s="24">
         <f>Supuestos!B24*Supuestos!B25</f>
         <v/>
       </c>
@@ -1524,7 +1525,7 @@
           <t>Total por mensaje</t>
         </is>
       </c>
-      <c r="B8" s="24">
+      <c r="B8" s="25">
         <f>SUM(B5:B7)</f>
         <v/>
       </c>
@@ -1536,7 +1537,7 @@
           <t>Costo por 100 mensajes</t>
         </is>
       </c>
-      <c r="B9" s="25">
+      <c r="B9" s="26">
         <f>B8*100</f>
         <v/>
       </c>
@@ -1548,7 +1549,7 @@
           <t>Precio mínimo por 100 mensajes para 60 % de margen</t>
         </is>
       </c>
-      <c r="B10" s="25">
+      <c r="B10" s="26">
         <f>B9/(1-0.6)</f>
         <v/>
       </c>
@@ -1703,31 +1704,31 @@
         <f>Supuestos!A6</f>
         <v/>
       </c>
-      <c r="B5" s="26">
+      <c r="B5" s="27">
         <f>Supuestos!B6</f>
         <v/>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="27">
         <f>B5*(1-Supuestos!$B$12)</f>
         <v/>
       </c>
-      <c r="D5" s="27">
+      <c r="D5" s="28">
         <f>Supuestos!C6</f>
         <v/>
       </c>
-      <c r="E5" s="27">
+      <c r="E5" s="28">
         <f>D5*Supuestos!E6</f>
         <v/>
       </c>
-      <c r="F5" s="26">
+      <c r="F5" s="27">
         <f>E5*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
-      <c r="G5" s="26">
+      <c r="G5" s="27">
         <f>D5*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
-      <c r="H5" s="26">
+      <c r="H5" s="27">
         <f>B5*(1-Supuestos!$B$26-Supuestos!$B$27)-F5</f>
         <v/>
       </c>
@@ -1735,7 +1736,7 @@
         <f>IF(B5=0,0,H5/B5)</f>
         <v/>
       </c>
-      <c r="J5" s="26">
+      <c r="J5" s="27">
         <f>C5*(1-Supuestos!$B$26-Supuestos!$B$27)-F5</f>
         <v/>
       </c>
@@ -1743,7 +1744,7 @@
         <f>IF(C5=0,0,J5/C5)</f>
         <v/>
       </c>
-      <c r="L5" s="26">
+      <c r="L5" s="27">
         <f>C5*(1-Supuestos!$B$26-Supuestos!$B$27)-G5</f>
         <v/>
       </c>
@@ -1753,31 +1754,31 @@
         <f>Supuestos!A7</f>
         <v/>
       </c>
-      <c r="B6" s="26">
+      <c r="B6" s="27">
         <f>Supuestos!B7</f>
         <v/>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="27">
         <f>B6*(1-Supuestos!$B$12)</f>
         <v/>
       </c>
-      <c r="D6" s="27">
+      <c r="D6" s="28">
         <f>Supuestos!C7</f>
         <v/>
       </c>
-      <c r="E6" s="27">
+      <c r="E6" s="28">
         <f>D6*Supuestos!E7</f>
         <v/>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="27">
         <f>E6*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
-      <c r="G6" s="26">
+      <c r="G6" s="27">
         <f>D6*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
-      <c r="H6" s="26">
+      <c r="H6" s="27">
         <f>B6*(1-Supuestos!$B$26-Supuestos!$B$27)-F6</f>
         <v/>
       </c>
@@ -1785,7 +1786,7 @@
         <f>IF(B6=0,0,H6/B6)</f>
         <v/>
       </c>
-      <c r="J6" s="26">
+      <c r="J6" s="27">
         <f>C6*(1-Supuestos!$B$26-Supuestos!$B$27)-F6</f>
         <v/>
       </c>
@@ -1793,7 +1794,7 @@
         <f>IF(C6=0,0,J6/C6)</f>
         <v/>
       </c>
-      <c r="L6" s="26">
+      <c r="L6" s="27">
         <f>C6*(1-Supuestos!$B$26-Supuestos!$B$27)-G6</f>
         <v/>
       </c>
@@ -1803,31 +1804,31 @@
         <f>Supuestos!A8</f>
         <v/>
       </c>
-      <c r="B7" s="26">
+      <c r="B7" s="27">
         <f>Supuestos!B8</f>
         <v/>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="27">
         <f>B7*(1-Supuestos!$B$12)</f>
         <v/>
       </c>
-      <c r="D7" s="27">
+      <c r="D7" s="28">
         <f>Supuestos!C8</f>
         <v/>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="28">
         <f>D7*Supuestos!E8</f>
         <v/>
       </c>
-      <c r="F7" s="26">
+      <c r="F7" s="27">
         <f>E7*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
-      <c r="G7" s="26">
+      <c r="G7" s="27">
         <f>D7*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
-      <c r="H7" s="26">
+      <c r="H7" s="27">
         <f>B7*(1-Supuestos!$B$26-Supuestos!$B$27)-F7</f>
         <v/>
       </c>
@@ -1835,7 +1836,7 @@
         <f>IF(B7=0,0,H7/B7)</f>
         <v/>
       </c>
-      <c r="J7" s="26">
+      <c r="J7" s="27">
         <f>C7*(1-Supuestos!$B$26-Supuestos!$B$27)-F7</f>
         <v/>
       </c>
@@ -1843,7 +1844,7 @@
         <f>IF(C7=0,0,J7/C7)</f>
         <v/>
       </c>
-      <c r="L7" s="26">
+      <c r="L7" s="27">
         <f>C7*(1-Supuestos!$B$26-Supuestos!$B$27)-G7</f>
         <v/>
       </c>
@@ -1868,22 +1869,22 @@
           <t>Recarga (+100 mensajes)</t>
         </is>
       </c>
-      <c r="B9" s="26">
+      <c r="B9" s="27">
         <f>Supuestos!B15</f>
         <v/>
       </c>
       <c r="C9" s="2" t="n"/>
-      <c r="D9" s="27">
+      <c r="D9" s="28">
         <f>Supuestos!B16</f>
         <v/>
       </c>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="n"/>
-      <c r="G9" s="26">
+      <c r="G9" s="27">
         <f>D9*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
-      <c r="H9" s="26">
+      <c r="H9" s="27">
         <f>B9*(1-Supuestos!$B$26-Supuestos!$B$27)-G9</f>
         <v/>
       </c>
@@ -1910,11 +1911,11 @@
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" s="26">
+      <c r="G10" s="27">
         <f>D10*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
-      <c r="H10" s="26">
+      <c r="H10" s="27">
         <f>B10*(1-Supuestos!$B$26-Supuestos!$B$27)-G10</f>
         <v/>
       </c>
@@ -1932,22 +1933,22 @@
           <t>Promedio ponderado por la mezcla de clientes</t>
         </is>
       </c>
-      <c r="B11" s="26">
+      <c r="B11" s="27">
         <f>SUMPRODUCT(B5:B7,Supuestos!D6:D8)</f>
         <v/>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="27">
         <f>SUMPRODUCT(C5:C7,Supuestos!D6:D8)</f>
         <v/>
       </c>
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
-      <c r="F11" s="26">
+      <c r="F11" s="27">
         <f>SUMPRODUCT(F5:F7,Supuestos!D6:D8)</f>
         <v/>
       </c>
       <c r="G11" s="2" t="n"/>
-      <c r="H11" s="26">
+      <c r="H11" s="27">
         <f>SUMPRODUCT(H5:H7,Supuestos!D6:D8)</f>
         <v/>
       </c>
@@ -1955,7 +1956,7 @@
         <f>IF(B11=0,0,H11/B11)</f>
         <v/>
       </c>
-      <c r="J11" s="26">
+      <c r="J11" s="27">
         <f>SUMPRODUCT(J5:J7,Supuestos!D6:D8)</f>
         <v/>
       </c>
@@ -1977,7 +1978,7 @@
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="n"/>
       <c r="G12" s="2" t="n"/>
-      <c r="H12" s="26">
+      <c r="H12" s="27">
         <f>Supuestos!B17*H9</f>
         <v/>
       </c>
@@ -2140,11 +2141,11 @@
           <t>Costos fijos al mes</t>
         </is>
       </c>
-      <c r="B5" s="26">
+      <c r="B5" s="27">
         <f>Supuestos!B36</f>
         <v/>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="27">
         <f>Supuestos!B36</f>
         <v/>
       </c>
@@ -2158,11 +2159,11 @@
           <t>Margen por cliente al mes (con recargas)</t>
         </is>
       </c>
-      <c r="B6" s="26">
+      <c r="B6" s="27">
         <f>'Margen por plan'!H13</f>
         <v/>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="27">
         <f>'Margen por plan'!J14</f>
         <v/>
       </c>
@@ -2176,11 +2177,11 @@
           <t>Clientes que pagan para cubrir los fijos</t>
         </is>
       </c>
-      <c r="B7" s="28">
+      <c r="B7" s="29">
         <f>IF(B6&lt;=0,"no se cubre",-INT(-B5/B6))</f>
         <v/>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="29">
         <f>IF(C6&lt;=0,"no se cubre",-INT(-C5/C6))</f>
         <v/>
       </c>
@@ -2194,11 +2195,11 @@
           <t>Ingreso mensual en el punto de equilibrio</t>
         </is>
       </c>
-      <c r="B8" s="26">
+      <c r="B8" s="27">
         <f>IF(ISNUMBER(B7),B7*'Margen por plan'!B11,0)</f>
         <v/>
       </c>
-      <c r="C8" s="26">
+      <c r="C8" s="27">
         <f>IF(ISNUMBER(C7),C7*'Margen por plan'!C11,0)</f>
         <v/>
       </c>
@@ -2262,19 +2263,19 @@
       <c r="A12" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="26">
+      <c r="B12" s="27">
         <f>A12*('Margen por plan'!$B$11+Supuestos!$B$17*Supuestos!$B$15)</f>
         <v/>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="27">
         <f>A12*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*('Costo por mensaje'!$B$5+'Costo por mensaje'!$B$7)+MAX(0,A12*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*Supuestos!$B$21-Supuestos!$B$23)*Supuestos!$B$22+B12*(Supuestos!$B$26+Supuestos!$B$27)</f>
         <v/>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="27">
         <f>Supuestos!$B$36</f>
         <v/>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="26">
         <f>B12-C12-D12</f>
         <v/>
       </c>
@@ -2287,19 +2288,19 @@
       <c r="A13" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="B13" s="26">
+      <c r="B13" s="27">
         <f>A13*('Margen por plan'!$B$11+Supuestos!$B$17*Supuestos!$B$15)</f>
         <v/>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="27">
         <f>A13*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*('Costo por mensaje'!$B$5+'Costo por mensaje'!$B$7)+MAX(0,A13*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*Supuestos!$B$21-Supuestos!$B$23)*Supuestos!$B$22+B13*(Supuestos!$B$26+Supuestos!$B$27)</f>
         <v/>
       </c>
-      <c r="D13" s="26">
+      <c r="D13" s="27">
         <f>Supuestos!$B$36</f>
         <v/>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="26">
         <f>B13-C13-D13</f>
         <v/>
       </c>
@@ -2312,19 +2313,19 @@
       <c r="A14" s="13" t="n">
         <v>50</v>
       </c>
-      <c r="B14" s="26">
+      <c r="B14" s="27">
         <f>A14*('Margen por plan'!$B$11+Supuestos!$B$17*Supuestos!$B$15)</f>
         <v/>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="27">
         <f>A14*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*('Costo por mensaje'!$B$5+'Costo por mensaje'!$B$7)+MAX(0,A14*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*Supuestos!$B$21-Supuestos!$B$23)*Supuestos!$B$22+B14*(Supuestos!$B$26+Supuestos!$B$27)</f>
         <v/>
       </c>
-      <c r="D14" s="26">
+      <c r="D14" s="27">
         <f>Supuestos!$B$36</f>
         <v/>
       </c>
-      <c r="E14" s="25">
+      <c r="E14" s="26">
         <f>B14-C14-D14</f>
         <v/>
       </c>
@@ -2337,19 +2338,19 @@
       <c r="A15" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="B15" s="26">
+      <c r="B15" s="27">
         <f>A15*('Margen por plan'!$B$11+Supuestos!$B$17*Supuestos!$B$15)</f>
         <v/>
       </c>
-      <c r="C15" s="26">
+      <c r="C15" s="27">
         <f>A15*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*('Costo por mensaje'!$B$5+'Costo por mensaje'!$B$7)+MAX(0,A15*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*Supuestos!$B$21-Supuestos!$B$23)*Supuestos!$B$22+B15*(Supuestos!$B$26+Supuestos!$B$27)</f>
         <v/>
       </c>
-      <c r="D15" s="26">
+      <c r="D15" s="27">
         <f>Supuestos!$B$36</f>
         <v/>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="26">
         <f>B15-C15-D15</f>
         <v/>
       </c>
@@ -2362,19 +2363,19 @@
       <c r="A16" s="13" t="n">
         <v>250</v>
       </c>
-      <c r="B16" s="26">
+      <c r="B16" s="27">
         <f>A16*('Margen por plan'!$B$11+Supuestos!$B$17*Supuestos!$B$15)</f>
         <v/>
       </c>
-      <c r="C16" s="26">
+      <c r="C16" s="27">
         <f>A16*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*('Costo por mensaje'!$B$5+'Costo por mensaje'!$B$7)+MAX(0,A16*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*Supuestos!$B$21-Supuestos!$B$23)*Supuestos!$B$22+B16*(Supuestos!$B$26+Supuestos!$B$27)</f>
         <v/>
       </c>
-      <c r="D16" s="26">
+      <c r="D16" s="27">
         <f>Supuestos!$B$36</f>
         <v/>
       </c>
-      <c r="E16" s="25">
+      <c r="E16" s="26">
         <f>B16-C16-D16</f>
         <v/>
       </c>
@@ -2387,19 +2388,19 @@
       <c r="A17" s="13" t="n">
         <v>500</v>
       </c>
-      <c r="B17" s="26">
+      <c r="B17" s="27">
         <f>A17*('Margen por plan'!$B$11+Supuestos!$B$17*Supuestos!$B$15)</f>
         <v/>
       </c>
-      <c r="C17" s="26">
+      <c r="C17" s="27">
         <f>A17*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*('Costo por mensaje'!$B$5+'Costo por mensaje'!$B$7)+MAX(0,A17*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*Supuestos!$B$21-Supuestos!$B$23)*Supuestos!$B$22+B17*(Supuestos!$B$26+Supuestos!$B$27)</f>
         <v/>
       </c>
-      <c r="D17" s="26">
+      <c r="D17" s="27">
         <f>Supuestos!$B$36</f>
         <v/>
       </c>
-      <c r="E17" s="25">
+      <c r="E17" s="26">
         <f>B17-C17-D17</f>
         <v/>
       </c>
@@ -2412,19 +2413,19 @@
       <c r="A18" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="B18" s="26">
+      <c r="B18" s="27">
         <f>A18*('Margen por plan'!$B$11+Supuestos!$B$17*Supuestos!$B$15)</f>
         <v/>
       </c>
-      <c r="C18" s="26">
+      <c r="C18" s="27">
         <f>A18*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*('Costo por mensaje'!$B$5+'Costo por mensaje'!$B$7)+MAX(0,A18*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*Supuestos!$B$21-Supuestos!$B$23)*Supuestos!$B$22+B18*(Supuestos!$B$26+Supuestos!$B$27)</f>
         <v/>
       </c>
-      <c r="D18" s="26">
+      <c r="D18" s="27">
         <f>Supuestos!$B$36</f>
         <v/>
       </c>
-      <c r="E18" s="25">
+      <c r="E18" s="26">
         <f>B18-C18-D18</f>
         <v/>
       </c>
@@ -2437,19 +2438,19 @@
       <c r="A19" s="13" t="n">
         <v>2000</v>
       </c>
-      <c r="B19" s="26">
+      <c r="B19" s="27">
         <f>A19*('Margen por plan'!$B$11+Supuestos!$B$17*Supuestos!$B$15)</f>
         <v/>
       </c>
-      <c r="C19" s="26">
+      <c r="C19" s="27">
         <f>A19*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*('Costo por mensaje'!$B$5+'Costo por mensaje'!$B$7)+MAX(0,A19*(SUMPRODUCT(Supuestos!$C$6:$C$8,Supuestos!$D$6:$D$8,Supuestos!$E$6:$E$8)+Supuestos!$B$17*Supuestos!$B$16)*Supuestos!$B$21-Supuestos!$B$23)*Supuestos!$B$22+B19*(Supuestos!$B$26+Supuestos!$B$27)</f>
         <v/>
       </c>
-      <c r="D19" s="26">
+      <c r="D19" s="27">
         <f>Supuestos!$B$36</f>
         <v/>
       </c>
-      <c r="E19" s="25">
+      <c r="E19" s="26">
         <f>B19-C19-D19</f>
         <v/>
       </c>
@@ -2532,11 +2533,11 @@
           <t>Clientes fundadores que pagan</t>
         </is>
       </c>
-      <c r="B5" s="27">
+      <c r="B5" s="28">
         <f>Supuestos!B14</f>
         <v/>
       </c>
-      <c r="C5" s="27">
+      <c r="C5" s="28">
         <f>Supuestos!B14</f>
         <v/>
       </c>
@@ -2552,11 +2553,11 @@
           <t>Personal</t>
         </is>
       </c>
-      <c r="B6" s="29">
+      <c r="B6" s="30">
         <f>B5*Supuestos!$D$6</f>
         <v/>
       </c>
-      <c r="C6" s="29">
+      <c r="C6" s="30">
         <f>C5*Supuestos!$D$6</f>
         <v/>
       </c>
@@ -2572,11 +2573,11 @@
           <t>Negocio</t>
         </is>
       </c>
-      <c r="B7" s="29">
+      <c r="B7" s="30">
         <f>B5*Supuestos!$D$7</f>
         <v/>
       </c>
-      <c r="C7" s="29">
+      <c r="C7" s="30">
         <f>C5*Supuestos!$D$7</f>
         <v/>
       </c>
@@ -2588,11 +2589,11 @@
           <t>Negocio Plus</t>
         </is>
       </c>
-      <c r="B8" s="29">
+      <c r="B8" s="30">
         <f>B5*Supuestos!$D$8</f>
         <v/>
       </c>
-      <c r="C8" s="29">
+      <c r="C8" s="30">
         <f>C5*Supuestos!$D$8</f>
         <v/>
       </c>
@@ -2604,11 +2605,11 @@
           <t>Ingreso de planes</t>
         </is>
       </c>
-      <c r="B9" s="26">
+      <c r="B9" s="27">
         <f>B6*'Margen por plan'!$C$5+B7*'Margen por plan'!$C$6+B8*'Margen por plan'!$C$7</f>
         <v/>
       </c>
-      <c r="C9" s="26">
+      <c r="C9" s="27">
         <f>C6*'Margen por plan'!$B$5+C7*'Margen por plan'!$B$6+C8*'Margen por plan'!$B$7</f>
         <v/>
       </c>
@@ -2620,11 +2621,11 @@
           <t>Ingreso de recargas</t>
         </is>
       </c>
-      <c r="B10" s="26">
+      <c r="B10" s="27">
         <f>B5*Supuestos!$B$17*Supuestos!$B$15</f>
         <v/>
       </c>
-      <c r="C10" s="26">
+      <c r="C10" s="27">
         <f>C5*Supuestos!$B$17*Supuestos!$B$15</f>
         <v/>
       </c>
@@ -2656,11 +2657,11 @@
           <t>Mensajes del mes</t>
         </is>
       </c>
-      <c r="B12" s="27">
+      <c r="B12" s="28">
         <f>B6*'Margen por plan'!$E$5+B7*'Margen por plan'!$E$6+B8*'Margen por plan'!$E$7+B5*Supuestos!$B$17*Supuestos!$B$16</f>
         <v/>
       </c>
-      <c r="C12" s="27">
+      <c r="C12" s="28">
         <f>C6*'Margen por plan'!$E$5+C7*'Margen por plan'!$E$6+C8*'Margen por plan'!$E$7+C5*Supuestos!$B$17*Supuestos!$B$16</f>
         <v/>
       </c>
@@ -2672,11 +2673,11 @@
           <t>Costo IA + voz</t>
         </is>
       </c>
-      <c r="B13" s="26">
+      <c r="B13" s="27">
         <f>B12*('Costo por mensaje'!$B$5+'Costo por mensaje'!$B$7)</f>
         <v/>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="27">
         <f>C12*('Costo por mensaje'!$B$5+'Costo por mensaje'!$B$7)</f>
         <v/>
       </c>
@@ -2688,11 +2689,11 @@
           <t>Costo Meta (después de 1.000 gratis)</t>
         </is>
       </c>
-      <c r="B14" s="26">
+      <c r="B14" s="27">
         <f>MAX(0,B12*Supuestos!$B$21-Supuestos!$B$23)*Supuestos!$B$22</f>
         <v/>
       </c>
-      <c r="C14" s="26">
+      <c r="C14" s="27">
         <f>MAX(0,C12*Supuestos!$B$21-Supuestos!$B$23)*Supuestos!$B$22</f>
         <v/>
       </c>
@@ -2704,11 +2705,11 @@
           <t>Comisiones e impuestos</t>
         </is>
       </c>
-      <c r="B15" s="26">
+      <c r="B15" s="27">
         <f>B11*(Supuestos!$B$26+Supuestos!$B$27)</f>
         <v/>
       </c>
-      <c r="C15" s="26">
+      <c r="C15" s="27">
         <f>C11*(Supuestos!$B$26+Supuestos!$B$27)</f>
         <v/>
       </c>
@@ -2720,11 +2721,11 @@
           <t>Costos fijos</t>
         </is>
       </c>
-      <c r="B16" s="26">
+      <c r="B16" s="27">
         <f>Supuestos!$B$36</f>
         <v/>
       </c>
-      <c r="C16" s="26">
+      <c r="C16" s="27">
         <f>Supuestos!$B$36</f>
         <v/>
       </c>
@@ -2768,7 +2769,7 @@
           <t>Ganancia acumulada en los meses de fundador</t>
         </is>
       </c>
-      <c r="B19" s="26">
+      <c r="B19" s="27">
         <f>B17*Supuestos!B13</f>
         <v/>
       </c>
@@ -2785,7 +2786,7 @@
           <t>Lo que se deja de ganar por el descuento (en esos meses)</t>
         </is>
       </c>
-      <c r="B20" s="26">
+      <c r="B20" s="27">
         <f>(C17-B17)*Supuestos!B13</f>
         <v/>
       </c>
@@ -3005,15 +3006,15 @@
           <t>Plan que eligen (precio fundador)</t>
         </is>
       </c>
-      <c r="B11" s="26">
+      <c r="B11" s="27">
         <f>'Margen por plan'!C5</f>
         <v/>
       </c>
-      <c r="C11" s="26">
+      <c r="C11" s="27">
         <f>'Margen por plan'!C6</f>
         <v/>
       </c>
-      <c r="D11" s="26">
+      <c r="D11" s="27">
         <f>'Margen por plan'!C5</f>
         <v/>
       </c>
@@ -3029,15 +3030,15 @@
           <t>Margen mensual por cliente que paga (fundador)</t>
         </is>
       </c>
-      <c r="B12" s="26">
+      <c r="B12" s="27">
         <f>'Margen por plan'!J5</f>
         <v/>
       </c>
-      <c r="C12" s="26">
+      <c r="C12" s="27">
         <f>'Margen por plan'!J6</f>
         <v/>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="27">
         <f>'Margen por plan'!J5</f>
         <v/>
       </c>
@@ -3053,15 +3054,15 @@
           <t>Mensajes incluidos en la prueba</t>
         </is>
       </c>
-      <c r="B13" s="27">
+      <c r="B13" s="28">
         <f>Supuestos!B40</f>
         <v/>
       </c>
-      <c r="C13" s="27">
+      <c r="C13" s="28">
         <f>Supuestos!B41</f>
         <v/>
       </c>
-      <c r="D13" s="27">
+      <c r="D13" s="28">
         <f>Supuestos!B40</f>
         <v/>
       </c>
@@ -3077,15 +3078,15 @@
           <t>Registrados</t>
         </is>
       </c>
-      <c r="B14" s="30">
+      <c r="B14" s="31">
         <f>B5*B6</f>
         <v/>
       </c>
-      <c r="C14" s="30">
+      <c r="C14" s="31">
         <f>C5*C6</f>
         <v/>
       </c>
-      <c r="D14" s="30">
+      <c r="D14" s="31">
         <f>D5*D6</f>
         <v/>
       </c>
@@ -3097,15 +3098,15 @@
           <t>Pruebas activas</t>
         </is>
       </c>
-      <c r="B15" s="30">
+      <c r="B15" s="31">
         <f>B14*B7</f>
         <v/>
       </c>
-      <c r="C15" s="30">
+      <c r="C15" s="31">
         <f>C14*C7</f>
         <v/>
       </c>
-      <c r="D15" s="30">
+      <c r="D15" s="31">
         <f>D14*D7</f>
         <v/>
       </c>
@@ -3117,15 +3118,15 @@
           <t>Pruebas inactivas</t>
         </is>
       </c>
-      <c r="B16" s="30">
+      <c r="B16" s="31">
         <f>B14-B15</f>
         <v/>
       </c>
-      <c r="C16" s="30">
+      <c r="C16" s="31">
         <f>C14-C15</f>
         <v/>
       </c>
-      <c r="D16" s="30">
+      <c r="D16" s="31">
         <f>D14-D15</f>
         <v/>
       </c>
@@ -3137,15 +3138,15 @@
           <t>Costo de las pruebas (Meta completo, con el tope)</t>
         </is>
       </c>
-      <c r="B17" s="26">
+      <c r="B17" s="27">
         <f>(B15*MIN(B8,B13)+B16*MIN(B9,B13))*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
-      <c r="C17" s="26">
+      <c r="C17" s="27">
         <f>(C15*MIN(C8,C13)+C16*MIN(C9,C13))*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
-      <c r="D17" s="26">
+      <c r="D17" s="27">
         <f>(D15*MIN(D8,D13)+D16*MIN(D9,D13))*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
@@ -3157,15 +3158,15 @@
           <t>Clientes que pagan</t>
         </is>
       </c>
-      <c r="B18" s="31">
+      <c r="B18" s="32">
         <f>B15*B10</f>
         <v/>
       </c>
-      <c r="C18" s="31">
+      <c r="C18" s="32">
         <f>C15*C10</f>
         <v/>
       </c>
-      <c r="D18" s="31">
+      <c r="D18" s="32">
         <f>D15*D10</f>
         <v/>
       </c>
@@ -3197,15 +3198,15 @@
           <t>Meses para recuperar el CAC</t>
         </is>
       </c>
-      <c r="B20" s="32">
+      <c r="B20" s="33">
         <f>IF(B12&lt;=0,0,B19/B12)</f>
         <v/>
       </c>
-      <c r="C20" s="32">
+      <c r="C20" s="33">
         <f>IF(C12&lt;=0,0,C19/C12)</f>
         <v/>
       </c>
-      <c r="D20" s="32">
+      <c r="D20" s="33">
         <f>IF(D12&lt;=0,0,D19/D12)</f>
         <v/>
       </c>
@@ -3217,15 +3218,15 @@
           <t>Ganancia mensual que aportan esos clientes</t>
         </is>
       </c>
-      <c r="B21" s="25">
+      <c r="B21" s="26">
         <f>B18*B12</f>
         <v/>
       </c>
-      <c r="C21" s="25">
+      <c r="C21" s="26">
         <f>C18*C12</f>
         <v/>
       </c>
-      <c r="D21" s="25">
+      <c r="D21" s="26">
         <f>D18*D12</f>
         <v/>
       </c>
@@ -3237,15 +3238,15 @@
           <t>Costo máximo de una prueba ($)</t>
         </is>
       </c>
-      <c r="B22" s="26">
+      <c r="B22" s="27">
         <f>B13*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
-      <c r="C22" s="26">
+      <c r="C22" s="27">
         <f>C13*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
-      <c r="D22" s="26">
+      <c r="D22" s="27">
         <f>D13*'Costo por mensaje'!$B$8</f>
         <v/>
       </c>
@@ -3261,7 +3262,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Lectura: el tipo de persona con el CAC más bajo y más clientes que pagan es a quien debes invitar primero. La prueba se mide en mensajes (100 Personal / 200 Negocio): el costo máximo de una prueba está en la fila 22.</t>
+          <t>Lectura: el tipo de persona con el CAC más bajo y más clientes que pagan es a quien debes invitar primero. La prueba es única: 14 días o 100 mensajes. El costo máximo de una prueba está en la fila 22 (~$2,13; ~$1 real mientras Meta regale las 1.000 respuestas del mes).</t>
         </is>
       </c>
       <c r="B24" s="2" t="n"/>
@@ -3397,34 +3398,34 @@
           <t>Movimientos anotados</t>
         </is>
       </c>
-      <c r="J4" s="33" t="inlineStr">
+      <c r="J4" s="34" t="inlineStr">
         <is>
           <t>IA por mensaje</t>
         </is>
       </c>
-      <c r="K4" s="33" t="inlineStr">
+      <c r="K4" s="34" t="inlineStr">
         <is>
           <t>Respuestas por mensaje</t>
         </is>
       </c>
-      <c r="L4" s="33" t="inlineStr">
+      <c r="L4" s="34" t="inlineStr">
         <is>
           <t>% notas de voz</t>
         </is>
       </c>
-      <c r="M4" s="33" t="inlineStr">
+      <c r="M4" s="34" t="inlineStr">
         <is>
           <t>Mensajes por día (activos)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="34" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>Autolavado (piloto 1)</t>
         </is>
       </c>
-      <c r="B5" s="34" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>Negocio</t>
         </is>
@@ -3453,18 +3454,18 @@
       <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="n"/>
-      <c r="M5" s="30">
+      <c r="M5" s="31">
         <f>IF(C5=0,0,D5/C5)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="34" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>Finanzas personales</t>
         </is>
       </c>
-      <c r="B6" s="34" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>Negocio</t>
         </is>
@@ -3493,18 +3494,18 @@
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="n"/>
-      <c r="M6" s="30">
+      <c r="M6" s="31">
         <f>IF(C6=0,0,D6/C6)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>Maria</t>
         </is>
       </c>
-      <c r="B7" s="34" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>Personal</t>
         </is>
@@ -3533,18 +3534,18 @@
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="n"/>
-      <c r="M7" s="30">
+      <c r="M7" s="31">
         <f>IF(C7=0,0,D7/C7)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="34" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>Finanzas Personales (sin uso)</t>
         </is>
       </c>
-      <c r="B8" s="34" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr">
         <is>
           <t>Negocio</t>
         </is>
@@ -3583,31 +3584,31 @@
       </c>
       <c r="B9" s="2" t="n"/>
       <c r="C9" s="2" t="n"/>
-      <c r="D9" s="28">
+      <c r="D9" s="29">
         <f>SUM(D5:D8)</f>
         <v/>
       </c>
-      <c r="E9" s="28">
+      <c r="E9" s="29">
         <f>SUM(E5:E8)</f>
         <v/>
       </c>
-      <c r="F9" s="28">
+      <c r="F9" s="29">
         <f>SUM(F5:F8)</f>
         <v/>
       </c>
-      <c r="G9" s="28">
+      <c r="G9" s="29">
         <f>SUM(G5:G8)</f>
         <v/>
       </c>
-      <c r="H9" s="24">
+      <c r="H9" s="25">
         <f>SUM(H5:H8)</f>
         <v/>
       </c>
-      <c r="I9" s="28">
+      <c r="I9" s="29">
         <f>SUM(I5:I8)</f>
         <v/>
       </c>
-      <c r="J9" s="24">
+      <c r="J9" s="25">
         <f>IF(D9=0,0,H9/D9)</f>
         <v/>
       </c>
@@ -3729,7 +3730,7 @@
       </c>
       <c r="B6" s="37" t="inlineStr">
         <is>
-          <t>Lotes de 10 a 15 por semana, no 100 de una vez: así puedes acompañar a cada uno, ver en /admin quién se activa y ajustar los textos de Rocco. La prueba se mide en mensajes: el peor caso es ~$2,10 por Personal (100) y ~$4,30 por Negocio (200).</t>
+          <t>Lotes de 10 a 15 por semana, no 100 de una vez: así puedes acompañar a cada uno, ver en /admin quién se activa y ajustar los textos de Rocco. La prueba es única (100 mensajes): el peor caso es ~$2,13 por persona; lo máximo en riesgo por tanda de 15 es ~$32.</t>
         </is>
       </c>
     </row>
@@ -3772,12 +3773,12 @@
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Prueba por mensajes y recargas</t>
+          <t>Prueba única y recargas</t>
         </is>
       </c>
       <c r="B10" s="37" t="inlineStr">
         <is>
-          <t>La prueba son 100 mensajes (Personal) o 200 (Negocio) en 14 días: unos 7 o 14 por día, más que el uso normal. Al llegar al tope del mes, quien quiere más compra recargas: +20 por $1 o +100 por $4. Las dos dejan más del 50 % de margen en el peor caso, así que el power user paga lo que usa y tu margen no cambia.</t>
+          <t>La prueba son 14 días o 100 mensajes para todos (unos 7 por día). Un negocio muy activo llega a 100 hacia el día 6: ese es el mejor momento para cobrar, no un problema. Al que valga la pena se le regalan +100 desde /admin. Al llegar al tope del mes, quien quiere más compra recargas: +20 por $1 o +100 por $4. Las dos dejan más del 50 % de margen en el peor caso, así que el power user paga lo que usa y tu margen no cambia.</t>
         </is>
       </c>
     </row>

</xml_diff>